<commit_message>
updating to reflect september fsa acreage report
</commit_message>
<xml_diff>
--- a/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
+++ b/data-raw/fsaCropAcreage/fsa_acreage_urls.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanturner/Library/CloudStorage/Dropbox-Personal/rfsa/data-raw/fsaCropAcreage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5EE7A08-587D-444E-8B46-B3F7E4B0C43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60035D67-2093-034D-B436-C6049B92DEF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="820" windowWidth="30240" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="150">
   <si>
     <t>raw_string</t>
   </si>
@@ -477,6 +477,12 @@
   </si>
   <si>
     <t>https://www.fsa.usda.gov/sites/default/files/2026-08/jhIRZDbkVKX5.zip</t>
+  </si>
+  <si>
+    <t>2026 acreage data as of September 11, 2026</t>
+  </si>
+  <si>
+    <t>https://www.fsa.usda.gov/sites/default/files/2026-09/06OAypAHYasf.zip</t>
   </si>
 </sst>
 </file>
@@ -833,7 +839,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.5" customWidth="1"/>
@@ -2341,6 +2347,26 @@
         <v>147</v>
       </c>
     </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>148</v>
+      </c>
+      <c r="B76">
+        <v>11</v>
+      </c>
+      <c r="C76">
+        <v>9</v>
+      </c>
+      <c r="D76">
+        <v>2026</v>
+      </c>
+      <c r="E76" s="2">
+        <v>46276</v>
+      </c>
+      <c r="F76" t="s">
+        <v>149</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F69">
     <sortCondition ref="E1:E69"/>

</xml_diff>